<commit_message>
Updated tests and demos.
</commit_message>
<xml_diff>
--- a/examples/informe_demo.xlsx
+++ b/examples/informe_demo.xlsx
@@ -178,7 +178,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.35</v>
+        <v>0.00</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -363,7 +363,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12.85</v>
+        <v>12.50</v>
       </c>
     </row>
     <row r="10">
@@ -415,58 +415,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transactions</t>
+          <t xml:space="preserve">Informes IBKR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">examples\demo_transactions.csv</t>
+          <t xml:space="preserve">examples/demo_ibkr_2025.csv</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Account</t>
+          <t xml:space="preserve">FX valores no EUR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">examples\demo_account.csv</t>
+          <t xml:space="preserve">ECB/BCE</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">FX mode solicitado</t>
+          <t xml:space="preserve">History end date</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">degiro</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FX mode aplicado</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">degiro</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">History end date</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-02-28</t>
         </is>
@@ -963,7 +939,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.85</v>
+        <v>10.50</v>
       </c>
     </row>
     <row r="4">
@@ -1003,7 +979,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10.85</v>
+        <v>10.50</v>
       </c>
     </row>
     <row r="8"/>
@@ -1114,7 +1090,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.35</v>
+        <v>0.00</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>

</xml_diff>